<commit_message>
data(topics): manual fit judgments for v3
</commit_message>
<xml_diff>
--- a/data/topics/topic_fit_check_v3.xlsx
+++ b/data/topics/topic_fit_check_v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ewallet-review-analysis\data\topics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B271AB-D8CE-42B1-8234-FFE3F881AA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514B98BB-E241-40FE-B407-FD0BD322548D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fit_check" sheetId="1" r:id="rId1"/>

</xml_diff>